<commit_message>
Actualizar plan de pruebas
</commit_message>
<xml_diff>
--- a/06_Plan_Pruebas.xlsx
+++ b/06_Plan_Pruebas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eldie\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eldie\Desktop\RQY1102_Grupo_D_ET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80CA9B8-B3E9-4B62-A5DE-699108E5C7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BBA2CA-675E-417E-892E-E63DE586D6F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3705" yWindow="2340" windowWidth="21600" windowHeight="11385" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Descripcion_Campos" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="139">
   <si>
     <t>DESCRIPCION DE CAMPOS</t>
   </si>
@@ -158,9 +158,6 @@
     <t>Fallido</t>
   </si>
   <si>
-    <t>Corregir validación</t>
-  </si>
-  <si>
     <t>CP-04</t>
   </si>
   <si>
@@ -416,9 +413,6 @@
     <t>Gestión de Comunidades</t>
   </si>
   <si>
-    <t>El sistema está incompleto, es importante agergar esas funciones.</t>
-  </si>
-  <si>
     <t>Cargar el Dashboard</t>
   </si>
   <si>
@@ -428,30 +422,18 @@
     <t>Información del Dashboard</t>
   </si>
   <si>
-    <t>Hay que agregar la información incompleta, cómo en CP--05.</t>
-  </si>
-  <si>
     <t>Activar una comunidad registrada anteriormente.</t>
   </si>
   <si>
     <t>Desactivar una comunidad y volver a activarla.</t>
   </si>
   <si>
-    <t>Error al querer volver a activar una comunidad desactivada.</t>
-  </si>
-  <si>
     <t>Visualizar comunidades en el Dashboard</t>
   </si>
   <si>
     <t>Legíbilidad del Dashboard</t>
   </si>
   <si>
-    <t>Se puede solucionar asignando más espacio al texto.</t>
-  </si>
-  <si>
-    <t>Puede resultar confuso, es importante tener la jerarquía clara.</t>
-  </si>
-  <si>
     <t>Uso de accesos directos</t>
   </si>
   <si>
@@ -461,9 +443,6 @@
     <t>Acceder a información detallada</t>
   </si>
   <si>
-    <t>Usa espacio de más en la pantalla y resulta confuso.</t>
-  </si>
-  <si>
     <t>Despliegue de acceso directo</t>
   </si>
   <si>
@@ -474,6 +453,9 @@
   </si>
   <si>
     <t>47.62%</t>
+  </si>
+  <si>
+    <t>Corregido en la última revisión</t>
   </si>
 </sst>
 </file>
@@ -1047,7 +1029,9 @@
       <c r="G4" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
@@ -1071,7 +1055,9 @@
       <c r="G5" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
@@ -1093,359 +1079,375 @@
         <v>37</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>39</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="D7" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>123</v>
-      </c>
       <c r="G7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="D8" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>46</v>
-      </c>
       <c r="G8" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>50</v>
-      </c>
       <c r="F9" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="E10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>55</v>
-      </c>
       <c r="G10" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="11" t="s">
-        <v>60</v>
-      </c>
       <c r="G11" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="11" t="s">
-        <v>65</v>
-      </c>
       <c r="G12" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>70</v>
-      </c>
       <c r="G13" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="F14" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>75</v>
-      </c>
       <c r="G14" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>80</v>
-      </c>
       <c r="G15" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="11"/>
+      <c r="H15" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>85</v>
-      </c>
       <c r="G16" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="C17" s="10" t="s">
+      <c r="D17" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="E17" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="F17" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="F17" s="11" t="s">
-        <v>90</v>
-      </c>
       <c r="G17" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H17" s="11"/>
+      <c r="H17" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="F18" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="F18" s="11" t="s">
-        <v>95</v>
-      </c>
       <c r="G18" s="11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="C19" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="E19" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="F19" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="F19" s="11" t="s">
-        <v>100</v>
-      </c>
       <c r="G19" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H19" s="11"/>
+      <c r="H19" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="E20" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="F20" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="F20" s="11" t="s">
-        <v>105</v>
-      </c>
       <c r="G20" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H20" s="11"/>
+      <c r="H20" s="11" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="12"/>
@@ -1476,20 +1478,20 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B4" s="5">
         <v>21</v>
@@ -1497,25 +1499,25 @@
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF(Registro_Pruebas!G4:G20,"Aprobado")</f>
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(Registro_Pruebas!G4:G20,"Fallido")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Registro_Pruebas!G4:G20,"Pendiente")</f>
@@ -1524,10 +1526,10 @@
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1548,7 +1550,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1556,7 +1558,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1564,7 +1566,7 @@
         <v>26</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1572,15 +1574,15 @@
         <v>38</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>118</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>